<commit_message>
Update: Ahmedabad-April-2026 by superadmin
</commit_message>
<xml_diff>
--- a/Ahmedabad-April-2026.xlsx
+++ b/Ahmedabad-April-2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aa30afadbe7955a4/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2023031\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="47" documentId="8_{9C2C097D-0996-4927-B700-EF5CEB99A3D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{82F745BA-CEEC-4594-9471-DA56E46AB7EA}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81C69893-7DBB-4B15-9AB2-A742ECB75BB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="APRIL26" sheetId="14" r:id="rId1"/>
@@ -388,9 +388,6 @@
     <t>Profit</t>
   </si>
   <si>
-    <t>Ahemdabad</t>
-  </si>
-  <si>
     <t>ERTIGA</t>
   </si>
   <si>
@@ -407,6 +404,9 @@
   </si>
   <si>
     <t>April</t>
+  </si>
+  <si>
+    <t>Ahmedabad</t>
   </si>
 </sst>
 </file>
@@ -513,7 +513,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -608,9 +608,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1001,38 +998,36 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A60573E7-0C10-47E9-84CF-CCBE31780A2B}">
   <dimension ref="A1:Z32"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="6.44140625" style="14" customWidth="1"/>
-    <col min="2" max="2" width="11.5546875" style="31" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.6640625" style="31" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.109375" style="31" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.5546875" style="31" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.33203125" style="31" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.77734375" style="14" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.33203125" style="14" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.5546875" style="14" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.33203125" style="14" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.5546875" style="14" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.44140625" style="14" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.5546875" style="14" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="17.6640625" style="14" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.44140625" style="14" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="16.21875" style="14" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.109375" style="14" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="17.21875" style="14" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18" style="14" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="13.77734375" style="14" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="15.77734375" style="14" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="18.77734375" style="14" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="8.5546875" style="14" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="14.44140625" style="14" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="10.21875" style="14" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="12.5546875" style="14" bestFit="1" customWidth="1"/>
-    <col min="27" max="16384" width="8.88671875" style="14"/>
+    <col min="1" max="1" width="11.140625" style="14" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.140625" style="31" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.85546875" style="31" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.42578125" style="31" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.140625" style="31" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.140625" style="31" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.28515625" style="14" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.140625" style="14" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17" style="14" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.85546875" style="14" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="12.5703125" style="14" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.7109375" style="14" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.42578125" style="14" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.42578125" style="14" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="16.7109375" style="14" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18" style="14" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.85546875" style="14" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="14" style="14" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="16" style="14" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="19" style="14" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="8.85546875" style="14" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="14.5703125" style="14" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="10.42578125" style="14" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="12.42578125" style="14" bestFit="1" customWidth="1"/>
+    <col min="27" max="16384" width="8.85546875" style="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:26" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>53</v>
       </c>
@@ -1112,15 +1107,15 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4">
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C2" s="35" t="s">
         <v>82</v>
+      </c>
+      <c r="C2" s="34" t="s">
+        <v>81</v>
       </c>
       <c r="D2" s="5">
         <v>2026</v>
@@ -1129,7 +1124,7 @@
         <v>3</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G2" s="8" t="s">
         <v>4</v>
@@ -1199,15 +1194,15 @@
         <v>15.823641986838853</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="14.4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:26" ht="15" x14ac:dyDescent="0.2">
       <c r="A3" s="4">
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C3" s="35" t="s">
         <v>82</v>
+      </c>
+      <c r="C3" s="34" t="s">
+        <v>81</v>
       </c>
       <c r="D3" s="5">
         <v>2026</v>
@@ -1216,7 +1211,7 @@
         <v>5</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G3" s="8" t="s">
         <v>4</v>
@@ -1286,15 +1281,15 @@
         <v>19.905141901124839</v>
       </c>
     </row>
-    <row r="4" spans="1:26" ht="14.4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:26" ht="15" x14ac:dyDescent="0.2">
       <c r="A4" s="4">
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C4" s="35" t="s">
         <v>82</v>
+      </c>
+      <c r="C4" s="34" t="s">
+        <v>81</v>
       </c>
       <c r="D4" s="5">
         <v>2026</v>
@@ -1303,7 +1298,7 @@
         <v>6</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G4" s="8" t="s">
         <v>4</v>
@@ -1373,15 +1368,15 @@
         <v>20.245186782068203</v>
       </c>
     </row>
-    <row r="5" spans="1:26" ht="14.4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:26" ht="15" x14ac:dyDescent="0.2">
       <c r="A5" s="4">
         <v>4</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C5" s="35" t="s">
         <v>82</v>
+      </c>
+      <c r="C5" s="34" t="s">
+        <v>81</v>
       </c>
       <c r="D5" s="5">
         <v>2026</v>
@@ -1390,7 +1385,7 @@
         <v>7</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G5" s="15" t="s">
         <v>8</v>
@@ -1460,15 +1455,15 @@
         <v>8.1698723442491463</v>
       </c>
     </row>
-    <row r="6" spans="1:26" ht="14.4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:26" ht="15" x14ac:dyDescent="0.2">
       <c r="A6" s="4">
         <v>5</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C6" s="35" t="s">
         <v>82</v>
+      </c>
+      <c r="C6" s="34" t="s">
+        <v>81</v>
       </c>
       <c r="D6" s="5">
         <v>2026</v>
@@ -1477,7 +1472,7 @@
         <v>9</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G6" s="15" t="s">
         <v>8</v>
@@ -1547,15 +1542,15 @@
         <v>2.0884702436905176</v>
       </c>
     </row>
-    <row r="7" spans="1:26" ht="14.4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:26" ht="15" x14ac:dyDescent="0.2">
       <c r="A7" s="4">
         <v>6</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C7" s="35" t="s">
         <v>82</v>
+      </c>
+      <c r="C7" s="34" t="s">
+        <v>81</v>
       </c>
       <c r="D7" s="5">
         <v>2026</v>
@@ -1634,15 +1629,15 @@
         <v>38.350624333572661</v>
       </c>
     </row>
-    <row r="8" spans="1:26" ht="14.4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:26" ht="15" x14ac:dyDescent="0.2">
       <c r="A8" s="4">
         <v>7</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C8" s="35" t="s">
         <v>82</v>
+      </c>
+      <c r="C8" s="34" t="s">
+        <v>81</v>
       </c>
       <c r="D8" s="5">
         <v>2026</v>
@@ -1721,15 +1716,15 @@
         <v>48.104992515425835</v>
       </c>
     </row>
-    <row r="9" spans="1:26" ht="14.4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:26" ht="15" x14ac:dyDescent="0.2">
       <c r="A9" s="4">
         <v>8</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C9" s="35" t="s">
         <v>82</v>
+      </c>
+      <c r="C9" s="34" t="s">
+        <v>81</v>
       </c>
       <c r="D9" s="5">
         <v>2026</v>
@@ -1808,15 +1803,15 @@
         <v>5.4123731137281492</v>
       </c>
     </row>
-    <row r="10" spans="1:26" ht="14.4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:26" ht="15" x14ac:dyDescent="0.2">
       <c r="A10" s="4">
         <v>9</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C10" s="35" t="s">
         <v>82</v>
+      </c>
+      <c r="C10" s="34" t="s">
+        <v>81</v>
       </c>
       <c r="D10" s="5">
         <v>2026</v>
@@ -1895,15 +1890,15 @@
         <v>-6.3856929594635723</v>
       </c>
     </row>
-    <row r="11" spans="1:26" ht="14.4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:26" ht="15" x14ac:dyDescent="0.2">
       <c r="A11" s="4">
         <v>10</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C11" s="35" t="s">
         <v>82</v>
+      </c>
+      <c r="C11" s="34" t="s">
+        <v>81</v>
       </c>
       <c r="D11" s="5">
         <v>2026</v>
@@ -1982,15 +1977,15 @@
         <v>38.292534696923219</v>
       </c>
     </row>
-    <row r="12" spans="1:26" ht="14.4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:26" ht="15" x14ac:dyDescent="0.2">
       <c r="A12" s="4">
         <v>11</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C12" s="35" t="s">
         <v>82</v>
+      </c>
+      <c r="C12" s="34" t="s">
+        <v>81</v>
       </c>
       <c r="D12" s="5">
         <v>2026</v>
@@ -2069,15 +2064,15 @@
         <v>3.6598955030913074</v>
       </c>
     </row>
-    <row r="13" spans="1:26" ht="14.4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:26" ht="15" x14ac:dyDescent="0.2">
       <c r="A13" s="4">
         <v>12</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C13" s="35" t="s">
         <v>82</v>
+      </c>
+      <c r="C13" s="34" t="s">
+        <v>81</v>
       </c>
       <c r="D13" s="5">
         <v>2026</v>
@@ -2156,15 +2151,15 @@
         <v>21.056999165360395</v>
       </c>
     </row>
-    <row r="14" spans="1:26" ht="14.4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:26" ht="15" x14ac:dyDescent="0.2">
       <c r="A14" s="4">
         <v>13</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C14" s="35" t="s">
         <v>82</v>
+      </c>
+      <c r="C14" s="34" t="s">
+        <v>81</v>
       </c>
       <c r="D14" s="5">
         <v>2026</v>
@@ -2243,15 +2238,15 @@
         <v>32.67875014127069</v>
       </c>
     </row>
-    <row r="15" spans="1:26" ht="14.4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:26" ht="15" x14ac:dyDescent="0.2">
       <c r="A15" s="4">
         <v>14</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C15" s="35" t="s">
         <v>82</v>
+      </c>
+      <c r="C15" s="34" t="s">
+        <v>81</v>
       </c>
       <c r="D15" s="5">
         <v>2026</v>
@@ -2329,15 +2324,15 @@
         <v>54.892616101185531</v>
       </c>
     </row>
-    <row r="16" spans="1:26" ht="14.4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:26" ht="15" x14ac:dyDescent="0.2">
       <c r="A16" s="4">
         <v>15</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C16" s="35" t="s">
         <v>82</v>
+      </c>
+      <c r="C16" s="34" t="s">
+        <v>81</v>
       </c>
       <c r="D16" s="5">
         <v>2026</v>
@@ -2416,15 +2411,15 @@
         <v>49.350210936717673</v>
       </c>
     </row>
-    <row r="17" spans="1:26" ht="14.4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:26" ht="15" x14ac:dyDescent="0.2">
       <c r="A17" s="4">
         <v>16</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C17" s="35" t="s">
         <v>82</v>
+      </c>
+      <c r="C17" s="34" t="s">
+        <v>81</v>
       </c>
       <c r="D17" s="5">
         <v>2026</v>
@@ -2503,15 +2498,15 @@
         <v>30.526866131512374</v>
       </c>
     </row>
-    <row r="18" spans="1:26" ht="14.4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:26" ht="15" x14ac:dyDescent="0.2">
       <c r="A18" s="4">
         <v>17</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C18" s="35" t="s">
         <v>82</v>
+      </c>
+      <c r="C18" s="34" t="s">
+        <v>81</v>
       </c>
       <c r="D18" s="5">
         <v>2026</v>
@@ -2590,15 +2585,15 @@
         <v>54.000208374788912</v>
       </c>
     </row>
-    <row r="19" spans="1:26" ht="14.4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:26" ht="15" x14ac:dyDescent="0.2">
       <c r="A19" s="4">
         <v>18</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C19" s="35" t="s">
         <v>82</v>
+      </c>
+      <c r="C19" s="34" t="s">
+        <v>81</v>
       </c>
       <c r="D19" s="5">
         <v>2026</v>
@@ -2677,15 +2672,15 @@
         <v>19.195100817168523</v>
       </c>
     </row>
-    <row r="20" spans="1:26" ht="14.4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:26" ht="15" x14ac:dyDescent="0.2">
       <c r="A20" s="4">
         <v>19</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C20" s="35" t="s">
         <v>82</v>
+      </c>
+      <c r="C20" s="34" t="s">
+        <v>81</v>
       </c>
       <c r="D20" s="5">
         <v>2026</v>
@@ -2764,15 +2759,15 @@
         <v>-7.4046426922730584</v>
       </c>
     </row>
-    <row r="21" spans="1:26" ht="14.4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:26" ht="15" x14ac:dyDescent="0.2">
       <c r="A21" s="4">
         <v>20</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C21" s="35" t="s">
         <v>82</v>
+      </c>
+      <c r="C21" s="34" t="s">
+        <v>81</v>
       </c>
       <c r="D21" s="5">
         <v>2026</v>
@@ -2851,15 +2846,15 @@
         <v>1.982860040878943</v>
       </c>
     </row>
-    <row r="22" spans="1:26" ht="14.4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:26" ht="15" x14ac:dyDescent="0.2">
       <c r="A22" s="4">
         <v>21</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C22" s="35" t="s">
         <v>82</v>
+      </c>
+      <c r="C22" s="34" t="s">
+        <v>81</v>
       </c>
       <c r="D22" s="5">
         <v>2026</v>
@@ -2938,15 +2933,15 @@
         <v>15.03489882481534</v>
       </c>
     </row>
-    <row r="23" spans="1:26" ht="14.4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:26" ht="15" x14ac:dyDescent="0.2">
       <c r="A23" s="4">
         <v>22</v>
       </c>
-      <c r="B23" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="C23" s="35" t="s">
+      <c r="B23" s="5" t="s">
         <v>82</v>
+      </c>
+      <c r="C23" s="34" t="s">
+        <v>81</v>
       </c>
       <c r="D23" s="5">
         <v>2026</v>
@@ -2954,8 +2949,8 @@
       <c r="E23" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="F23" s="34" t="s">
-        <v>79</v>
+      <c r="F23" s="33" t="s">
+        <v>78</v>
       </c>
       <c r="G23" s="8" t="s">
         <v>37</v>
@@ -3025,15 +3020,15 @@
         <v>-39.047288534532704</v>
       </c>
     </row>
-    <row r="24" spans="1:26" ht="14.4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:26" ht="15" x14ac:dyDescent="0.2">
       <c r="A24" s="4">
         <v>23</v>
       </c>
-      <c r="B24" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="C24" s="35" t="s">
+      <c r="B24" s="5" t="s">
         <v>82</v>
+      </c>
+      <c r="C24" s="34" t="s">
+        <v>81</v>
       </c>
       <c r="D24" s="5">
         <v>2026</v>
@@ -3041,8 +3036,8 @@
       <c r="E24" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="F24" s="34" t="s">
-        <v>79</v>
+      <c r="F24" s="33" t="s">
+        <v>78</v>
       </c>
       <c r="G24" s="8" t="s">
         <v>37</v>
@@ -3112,15 +3107,15 @@
         <v>-79.560325354980833</v>
       </c>
     </row>
-    <row r="25" spans="1:26" ht="14.4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:26" ht="15" x14ac:dyDescent="0.2">
       <c r="A25" s="4">
         <v>24</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C25" s="35" t="s">
         <v>82</v>
+      </c>
+      <c r="C25" s="34" t="s">
+        <v>81</v>
       </c>
       <c r="D25" s="5">
         <v>2026</v>
@@ -3199,15 +3194,15 @@
         <v>68.678130110322613</v>
       </c>
     </row>
-    <row r="26" spans="1:26" ht="14.4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:26" ht="15" x14ac:dyDescent="0.2">
       <c r="A26" s="4">
         <v>25</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C26" s="35" t="s">
         <v>82</v>
+      </c>
+      <c r="C26" s="34" t="s">
+        <v>81</v>
       </c>
       <c r="D26" s="5">
         <v>2026</v>
@@ -3216,7 +3211,7 @@
         <v>42</v>
       </c>
       <c r="F26" s="17" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G26" s="27" t="s">
         <v>43</v>
@@ -3285,15 +3280,15 @@
         <v>15.435636891226537</v>
       </c>
     </row>
-    <row r="27" spans="1:26" ht="14.4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:26" ht="15" x14ac:dyDescent="0.2">
       <c r="A27" s="4">
         <v>26</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C27" s="35" t="s">
         <v>82</v>
+      </c>
+      <c r="C27" s="34" t="s">
+        <v>81</v>
       </c>
       <c r="D27" s="5">
         <v>2026</v>
@@ -3302,7 +3297,7 @@
         <v>44</v>
       </c>
       <c r="F27" s="17" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G27" s="9" t="s">
         <v>45</v>
@@ -3372,15 +3367,15 @@
         <v>33.037168500984016</v>
       </c>
     </row>
-    <row r="28" spans="1:26" ht="14.4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:26" ht="15" x14ac:dyDescent="0.2">
       <c r="A28" s="4">
         <v>27</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C28" s="35" t="s">
         <v>82</v>
+      </c>
+      <c r="C28" s="34" t="s">
+        <v>81</v>
       </c>
       <c r="D28" s="5">
         <v>2026</v>
@@ -3389,7 +3384,7 @@
         <v>46</v>
       </c>
       <c r="F28" s="17" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G28" s="9" t="s">
         <v>47</v>
@@ -3459,15 +3454,15 @@
         <v>28.288534938119867</v>
       </c>
     </row>
-    <row r="29" spans="1:26" ht="14.4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:26" ht="15" x14ac:dyDescent="0.2">
       <c r="A29" s="4">
         <v>28</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C29" s="35" t="s">
         <v>82</v>
+      </c>
+      <c r="C29" s="34" t="s">
+        <v>81</v>
       </c>
       <c r="D29" s="5">
         <v>2026</v>
@@ -3476,7 +3471,7 @@
         <v>48</v>
       </c>
       <c r="F29" s="17" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G29" s="29" t="s">
         <v>49</v>
@@ -3546,15 +3541,15 @@
         <v>34.786780750757494</v>
       </c>
     </row>
-    <row r="30" spans="1:26" ht="14.4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:26" ht="15" x14ac:dyDescent="0.2">
       <c r="A30" s="4">
         <v>29</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C30" s="35" t="s">
         <v>82</v>
+      </c>
+      <c r="C30" s="34" t="s">
+        <v>81</v>
       </c>
       <c r="D30" s="5">
         <v>2026</v>
@@ -3563,7 +3558,7 @@
         <v>50</v>
       </c>
       <c r="F30" s="17" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G30" s="29" t="s">
         <v>45</v>
@@ -3634,15 +3629,15 @@
         <v>12.552578922725131</v>
       </c>
     </row>
-    <row r="31" spans="1:26" ht="14.4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:26" ht="15" x14ac:dyDescent="0.2">
       <c r="A31" s="4">
         <v>30</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C31" s="35" t="s">
         <v>82</v>
+      </c>
+      <c r="C31" s="34" t="s">
+        <v>81</v>
       </c>
       <c r="D31" s="5">
         <v>2026</v>
@@ -3651,7 +3646,7 @@
         <v>51</v>
       </c>
       <c r="F31" s="17" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G31" s="29" t="s">
         <v>52</v>
@@ -3722,7 +3717,7 @@
         <v>20.032518801655325</v>
       </c>
     </row>
-    <row r="32" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:26" x14ac:dyDescent="0.2">
       <c r="F32" s="5"/>
       <c r="H32" s="32"/>
       <c r="T32" s="32"/>
@@ -3732,17 +3727,22 @@
   <autoFilter ref="A1:Z31" xr:uid="{A60573E7-0C10-47E9-84CF-CCBE31780A2B}"/>
   <phoneticPr fontId="9" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;10&amp;K000000 Revvity Proprietary Information</oddFooter>
+  </headerFooter>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="32a854ad-91b1-449d-ac0d-217ac9c33903">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="358f3261-8c6f-476a-b02c-56882718635b" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4001,20 +4001,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="32a854ad-91b1-449d-ac0d-217ac9c33903">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="358f3261-8c6f-476a-b02c-56882718635b" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ACD769C3-07DD-4F20-BF9C-C3BA66D61815}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{55DC610F-D2CB-44E4-9CF3-16B359AF01B2}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="32a854ad-91b1-449d-ac0d-217ac9c33903"/>
+    <ds:schemaRef ds:uri="358f3261-8c6f-476a-b02c-56882718635b"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -4039,12 +4040,15 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{55DC610F-D2CB-44E4-9CF3-16B359AF01B2}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ACD769C3-07DD-4F20-BF9C-C3BA66D61815}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="32a854ad-91b1-449d-ac0d-217ac9c33903"/>
-    <ds:schemaRef ds:uri="358f3261-8c6f-476a-b02c-56882718635b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{a1b582e8-0077-416f-9765-e019f2ce0792}" enabled="1" method="Standard" siteId="{66a92d0f-8ca8-403c-84e6-5503c5643994}" contentBits="2" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>